<commit_message>
Route all log files to logs/ subfolder, clean up stale JSON artifacts
- Switch asd_risk_classifier.py and OAIC_dashboard_scraper.py from
  hardcoded FileHandler paths to shared setup_logging() with logs/ prefix
- Add missing Path import to logging_config.py
- Delete 19 raw OAIC statistics files (consolidated via cleanup_oaic_data.py)
- Delete migration_report and oaic_screenshots artifacts
- Regenerate dashboard and risk matrices

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -503,10 +503,10 @@
       <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>9</v>
@@ -522,20 +522,20 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -545,19 +545,19 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
     </row>
@@ -570,9 +570,7 @@
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
     </row>
@@ -584,15 +582,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr"/>
       <c r="C6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="G6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
@@ -602,19 +602,19 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Add pipeline documentation, incremental dedup, force-dedup flag, dashboard fixes
- Add comprehensive docs/ directory with 9 detailed specification documents
  covering all pipeline stages (data sources, discovery, scraping, filtering,
  enrichment, deduplication, ASD classification, dashboard generation, data
  dictionary)
- Refactor global deduplication to support incremental mode (only process new
  events) with --force-dedup flag for full rebuilds
- Add tqdm progress bars to deduplication replacing manual log-every-100 pattern
- Fix missing asd_risk_previous key in dashboard data dictionary
- Update dashboard and risk matrix Excel outputs with latest data

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -509,7 +509,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>1</v>
@@ -522,17 +522,17 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>215</v>
+        <v>183</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>2</v>
@@ -548,16 +548,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
     </row>
@@ -570,7 +570,9 @@
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
     </row>
@@ -580,15 +582,17 @@
           <t>Low-level malicious attack</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr"/>
+      <c r="B6" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="C6" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>2</v>
@@ -602,22 +606,22 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>